<commit_message>
fix(deliverability): update 100 intent tracker and CRM with verified delivery vs bounced audit
</commit_message>
<xml_diff>
--- a/data/100_INTENT_LEADS_OMNICHANNEL_TRACKER.xlsx
+++ b/data/100_INTENT_LEADS_OMNICHANNEL_TRACKER.xlsx
@@ -48,7 +48,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -79,6 +79,18 @@
         <bgColor rgb="00FEF2F2"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D1E7DD"/>
+        <bgColor rgb="00D1E7DD"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F8D7DA"/>
+        <bgColor rgb="00F8D7DA"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -106,7 +118,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -122,6 +134,12 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -851,9 +869,9 @@
           <t>High-intent signal: actively hiring Medical Receptionist. Validated website and LinkedIn. Requires Clay enrichment for verified email.</t>
         </is>
       </c>
-      <c r="AF2" s="3" t="inlineStr">
-        <is>
-          <t>✔ Sent</t>
+      <c r="AF2" s="6" t="inlineStr">
+        <is>
+          <t>✔ Delivered (Clean Inbox)</t>
         </is>
       </c>
       <c r="AG2" s="4" t="inlineStr">
@@ -1019,9 +1037,9 @@
           <t>High-intent signal: actively hiring Medical Receptionist. Validated website and LinkedIn. Requires Clay enrichment for verified email.</t>
         </is>
       </c>
-      <c r="AF3" s="3" t="inlineStr">
-        <is>
-          <t>✔ Sent</t>
+      <c r="AF3" s="7" t="inlineStr">
+        <is>
+          <t>❌ Bounced (Address Not Found)</t>
         </is>
       </c>
       <c r="AG3" s="4" t="inlineStr">
@@ -1187,9 +1205,9 @@
           <t>High-intent signal: actively hiring Real Estate Telecaller / Lead Caller. Validated website and LinkedIn. Requires Clay enrichment for verified email.</t>
         </is>
       </c>
-      <c r="AF4" s="3" t="inlineStr">
-        <is>
-          <t>✔ Sent</t>
+      <c r="AF4" s="6" t="inlineStr">
+        <is>
+          <t>✔ Delivered (Clean Inbox)</t>
         </is>
       </c>
       <c r="AG4" s="4" t="inlineStr">
@@ -1355,9 +1373,9 @@
           <t>High-intent signal: actively hiring Medical Receptionist. Validated website and LinkedIn. Requires Clay enrichment for verified email.</t>
         </is>
       </c>
-      <c r="AF5" s="3" t="inlineStr">
-        <is>
-          <t>✔ Sent</t>
+      <c r="AF5" s="6" t="inlineStr">
+        <is>
+          <t>✔ Delivered (Clean Inbox)</t>
         </is>
       </c>
       <c r="AG5" s="4" t="inlineStr">
@@ -1523,9 +1541,9 @@
           <t>High-intent signal: actively hiring Medical Receptionist Dermatology. Validated website and LinkedIn. Requires Clay enrichment for verified email.</t>
         </is>
       </c>
-      <c r="AF6" s="3" t="inlineStr">
-        <is>
-          <t>✔ Sent</t>
+      <c r="AF6" s="7" t="inlineStr">
+        <is>
+          <t>❌ Bounced (Address Not Found)</t>
         </is>
       </c>
       <c r="AG6" s="4" t="inlineStr">
@@ -1691,9 +1709,9 @@
           <t>High-intent signal: actively hiring Surgical New Patient Coordinator. Validated website and LinkedIn. Requires Clay enrichment for verified email.</t>
         </is>
       </c>
-      <c r="AF7" s="3" t="inlineStr">
-        <is>
-          <t>✔ Sent</t>
+      <c r="AF7" s="7" t="inlineStr">
+        <is>
+          <t>❌ Bounced (Address Not Found)</t>
         </is>
       </c>
       <c r="AG7" s="4" t="inlineStr">
@@ -2195,9 +2213,9 @@
           <t>High-intent signal: actively hiring Front Desk Receptionist / Sales Coordinator. Validated website and LinkedIn. Requires Clay enrichment for verified email.</t>
         </is>
       </c>
-      <c r="AF10" s="3" t="inlineStr">
-        <is>
-          <t>✔ Sent</t>
+      <c r="AF10" s="6" t="inlineStr">
+        <is>
+          <t>✔ Delivered (Clean Inbox)</t>
         </is>
       </c>
       <c r="AG10" s="4" t="inlineStr">
@@ -2363,9 +2381,9 @@
           <t>High-intent signal: actively hiring Medical Receptionist. Validated website and LinkedIn. Requires Clay enrichment for verified email.</t>
         </is>
       </c>
-      <c r="AF11" s="3" t="inlineStr">
-        <is>
-          <t>✔ Sent</t>
+      <c r="AF11" s="7" t="inlineStr">
+        <is>
+          <t>❌ Bounced (Address Not Found)</t>
         </is>
       </c>
       <c r="AG11" s="4" t="inlineStr">
@@ -2531,9 +2549,9 @@
           <t>High-intent signal: actively hiring Medical Receptionist. Validated website and LinkedIn. Requires Clay enrichment for verified email.</t>
         </is>
       </c>
-      <c r="AF12" s="3" t="inlineStr">
-        <is>
-          <t>✔ Sent</t>
+      <c r="AF12" s="6" t="inlineStr">
+        <is>
+          <t>✔ Delivered (Clean Inbox)</t>
         </is>
       </c>
       <c r="AG12" s="4" t="inlineStr">
@@ -2699,9 +2717,9 @@
           <t>High-intent signal: actively hiring Front Desk Agent. Validated website and LinkedIn. Requires Clay enrichment for verified email.</t>
         </is>
       </c>
-      <c r="AF13" s="3" t="inlineStr">
-        <is>
-          <t>✔ Sent</t>
+      <c r="AF13" s="6" t="inlineStr">
+        <is>
+          <t>✔ Delivered (Clean Inbox)</t>
         </is>
       </c>
       <c r="AG13" s="4" t="inlineStr">
@@ -2867,9 +2885,9 @@
           <t>High-intent signal: actively hiring Medical Receptionist (Urgent Care). Validated website and LinkedIn. Requires Clay enrichment for verified email.</t>
         </is>
       </c>
-      <c r="AF14" s="3" t="inlineStr">
-        <is>
-          <t>✔ Sent</t>
+      <c r="AF14" s="7" t="inlineStr">
+        <is>
+          <t>❌ Bounced (Address Not Found)</t>
         </is>
       </c>
       <c r="AG14" s="4" t="inlineStr">
@@ -3035,9 +3053,9 @@
           <t>High-intent signal: actively hiring Medical Receptionist. Validated website and LinkedIn. Requires Clay enrichment for verified email.</t>
         </is>
       </c>
-      <c r="AF15" s="3" t="inlineStr">
-        <is>
-          <t>✔ Sent</t>
+      <c r="AF15" s="7" t="inlineStr">
+        <is>
+          <t>❌ Bounced (Address Not Found)</t>
         </is>
       </c>
       <c r="AG15" s="4" t="inlineStr">
@@ -3203,9 +3221,9 @@
           <t>High-intent signal: actively hiring Front Desk Salon Coordinator. Validated website and LinkedIn. Requires Clay enrichment for verified email.</t>
         </is>
       </c>
-      <c r="AF16" s="3" t="inlineStr">
-        <is>
-          <t>✔ Sent</t>
+      <c r="AF16" s="6" t="inlineStr">
+        <is>
+          <t>✔ Delivered (Clean Inbox)</t>
         </is>
       </c>
       <c r="AG16" s="4" t="inlineStr">
@@ -3371,9 +3389,9 @@
           <t>High-intent signal: actively hiring Front Desk Receptionist. Validated website and LinkedIn. Requires Clay enrichment for verified email.</t>
         </is>
       </c>
-      <c r="AF17" s="3" t="inlineStr">
-        <is>
-          <t>✔ Sent</t>
+      <c r="AF17" s="7" t="inlineStr">
+        <is>
+          <t>❌ Bounced (Address Not Found)</t>
         </is>
       </c>
       <c r="AG17" s="4" t="inlineStr">
@@ -3539,9 +3557,9 @@
           <t>High-intent signal: actively hiring Front Desk Coordinator + Social Media. Validated website and LinkedIn. Requires Clay enrichment for verified email.</t>
         </is>
       </c>
-      <c r="AF18" s="3" t="inlineStr">
-        <is>
-          <t>✔ Sent</t>
+      <c r="AF18" s="7" t="inlineStr">
+        <is>
+          <t>❌ Bounced (Address Not Found)</t>
         </is>
       </c>
       <c r="AG18" s="4" t="inlineStr">
@@ -3707,9 +3725,9 @@
           <t>High-intent signal: actively hiring Coordinator, Talent Acquisition. Validated website and LinkedIn. Requires Clay enrichment for verified email.</t>
         </is>
       </c>
-      <c r="AF19" s="3" t="inlineStr">
-        <is>
-          <t>✔ Sent</t>
+      <c r="AF19" s="7" t="inlineStr">
+        <is>
+          <t>❌ Bounced (Address Not Found)</t>
         </is>
       </c>
       <c r="AG19" s="4" t="inlineStr">
@@ -3875,9 +3893,9 @@
           <t>High-intent signal: actively hiring Temporary Talent Acquisition Specialist. Validated website and LinkedIn. Requires Clay enrichment for verified email.</t>
         </is>
       </c>
-      <c r="AF20" s="3" t="inlineStr">
-        <is>
-          <t>✔ Sent</t>
+      <c r="AF20" s="6" t="inlineStr">
+        <is>
+          <t>✔ Delivered (Clean Inbox)</t>
         </is>
       </c>
       <c r="AG20" s="4" t="inlineStr">
@@ -4043,9 +4061,9 @@
           <t>High-intent signal: actively hiring Salon Coordinator / Front Desk Receptionist. Validated website and LinkedIn. Requires Clay enrichment for verified email.</t>
         </is>
       </c>
-      <c r="AF21" s="3" t="inlineStr">
-        <is>
-          <t>✔ Sent</t>
+      <c r="AF21" s="6" t="inlineStr">
+        <is>
+          <t>✔ Delivered (Clean Inbox)</t>
         </is>
       </c>
       <c r="AG21" s="4" t="inlineStr">
@@ -4211,9 +4229,9 @@
           <t>High-intent signal: actively hiring Talent Acquisition Partner - Global E-Commerce. Validated website and LinkedIn. Requires Clay enrichment for verified email.</t>
         </is>
       </c>
-      <c r="AF22" s="3" t="inlineStr">
-        <is>
-          <t>✔ Sent</t>
+      <c r="AF22" s="7" t="inlineStr">
+        <is>
+          <t>❌ Bounced (Address Not Found)</t>
         </is>
       </c>
       <c r="AG22" s="4" t="inlineStr">
@@ -4379,9 +4397,9 @@
           <t>High-intent signal: actively hiring Senior Talent Acquisition Specialist. Validated website and LinkedIn. Requires Clay enrichment for verified email.</t>
         </is>
       </c>
-      <c r="AF23" s="3" t="inlineStr">
-        <is>
-          <t>✔ Sent</t>
+      <c r="AF23" s="7" t="inlineStr">
+        <is>
+          <t>❌ Bounced (Address Not Found)</t>
         </is>
       </c>
       <c r="AG23" s="4" t="inlineStr">
@@ -4547,9 +4565,9 @@
           <t>High-intent signal: actively hiring Senior Talent Acquisition Sourcing Specialist. Validated website and LinkedIn. Requires Clay enrichment for verified email.</t>
         </is>
       </c>
-      <c r="AF24" s="3" t="inlineStr">
-        <is>
-          <t>✔ Sent</t>
+      <c r="AF24" s="7" t="inlineStr">
+        <is>
+          <t>❌ Bounced (Address Not Found)</t>
         </is>
       </c>
       <c r="AG24" s="4" t="inlineStr">
@@ -4715,9 +4733,9 @@
           <t>High-intent signal: actively hiring Talent Acquisition Sourcing Specialist. Validated website and LinkedIn. Requires Clay enrichment for verified email.</t>
         </is>
       </c>
-      <c r="AF25" s="3" t="inlineStr">
-        <is>
-          <t>✔ Sent</t>
+      <c r="AF25" s="6" t="inlineStr">
+        <is>
+          <t>✔ Delivered (Clean Inbox)</t>
         </is>
       </c>
       <c r="AG25" s="4" t="inlineStr">
@@ -4883,9 +4901,9 @@
           <t>High-intent signal: actively hiring Front Desk Coordinator/Receptionist. Validated website and LinkedIn. Requires Clay enrichment for verified email.</t>
         </is>
       </c>
-      <c r="AF26" s="3" t="inlineStr">
-        <is>
-          <t>✔ Sent</t>
+      <c r="AF26" s="7" t="inlineStr">
+        <is>
+          <t>❌ Bounced (Address Not Found)</t>
         </is>
       </c>
       <c r="AG26" s="4" t="inlineStr">
@@ -5051,9 +5069,9 @@
           <t>High-intent signal: actively hiring Spa/Salon Front Desk Coordinator &amp; Sales Advisor. Validated website and LinkedIn. Requires Clay enrichment for verified email.</t>
         </is>
       </c>
-      <c r="AF27" s="3" t="inlineStr">
-        <is>
-          <t>✔ Sent</t>
+      <c r="AF27" s="6" t="inlineStr">
+        <is>
+          <t>✔ Delivered (Clean Inbox)</t>
         </is>
       </c>
       <c r="AG27" s="4" t="inlineStr">
@@ -5219,9 +5237,9 @@
           <t>High-intent signal: actively hiring Talent Acquisition Specialist. Validated website and LinkedIn. Requires Clay enrichment for verified email.</t>
         </is>
       </c>
-      <c r="AF28" s="3" t="inlineStr">
-        <is>
-          <t>✔ Sent</t>
+      <c r="AF28" s="6" t="inlineStr">
+        <is>
+          <t>✔ Delivered (Clean Inbox)</t>
         </is>
       </c>
       <c r="AG28" s="4" t="inlineStr">
@@ -5387,9 +5405,9 @@
           <t>High-intent signal: actively hiring Front Desk Associate. Validated website and LinkedIn. Requires Clay enrichment for verified email.</t>
         </is>
       </c>
-      <c r="AF29" s="3" t="inlineStr">
-        <is>
-          <t>✔ Sent</t>
+      <c r="AF29" s="6" t="inlineStr">
+        <is>
+          <t>✔ Delivered (Clean Inbox)</t>
         </is>
       </c>
       <c r="AG29" s="4" t="inlineStr">
@@ -5555,9 +5573,9 @@
           <t>High-intent signal: actively hiring Front Desk Coordinator Receptionist. Validated website and LinkedIn. Requires Clay enrichment for verified email.</t>
         </is>
       </c>
-      <c r="AF30" s="3" t="inlineStr">
-        <is>
-          <t>✔ Sent</t>
+      <c r="AF30" s="7" t="inlineStr">
+        <is>
+          <t>❌ Bounced (Address Not Found)</t>
         </is>
       </c>
       <c r="AG30" s="4" t="inlineStr">
@@ -5723,9 +5741,9 @@
           <t>High-intent signal: actively hiring Front Desk Coordinator/Receptionist. Validated website and LinkedIn. Requires Clay enrichment for verified email.</t>
         </is>
       </c>
-      <c r="AF31" s="3" t="inlineStr">
-        <is>
-          <t>✔ Sent</t>
+      <c r="AF31" s="7" t="inlineStr">
+        <is>
+          <t>❌ Bounced (Address Not Found)</t>
         </is>
       </c>
       <c r="AG31" s="4" t="inlineStr">
@@ -5891,9 +5909,9 @@
           <t>High-intent signal: actively hiring Talent Acquisition Specialist - Healthcare. Validated website and LinkedIn. Requires Clay enrichment for verified email.</t>
         </is>
       </c>
-      <c r="AF32" s="3" t="inlineStr">
-        <is>
-          <t>✔ Sent</t>
+      <c r="AF32" s="7" t="inlineStr">
+        <is>
+          <t>❌ Bounced (Address Not Found)</t>
         </is>
       </c>
       <c r="AG32" s="4" t="inlineStr">
@@ -6059,9 +6077,9 @@
           <t>High-intent signal: actively hiring Talent Acquisition Partner. Validated website and LinkedIn. Requires Clay enrichment for verified email.</t>
         </is>
       </c>
-      <c r="AF33" s="3" t="inlineStr">
-        <is>
-          <t>✔ Sent</t>
+      <c r="AF33" s="7" t="inlineStr">
+        <is>
+          <t>❌ Bounced (Address Not Found)</t>
         </is>
       </c>
       <c r="AG33" s="4" t="inlineStr">
@@ -6227,9 +6245,9 @@
           <t>High-intent signal: actively hiring Talent Acquisition Partner. Validated website and LinkedIn. Requires Clay enrichment for verified email.</t>
         </is>
       </c>
-      <c r="AF34" s="3" t="inlineStr">
-        <is>
-          <t>✔ Sent</t>
+      <c r="AF34" s="7" t="inlineStr">
+        <is>
+          <t>❌ Bounced (Address Not Found)</t>
         </is>
       </c>
       <c r="AG34" s="4" t="inlineStr">
@@ -6395,9 +6413,9 @@
           <t>High-intent signal: actively hiring Talent Acquisition Specialist. Validated website and LinkedIn. Requires Clay enrichment for verified email.</t>
         </is>
       </c>
-      <c r="AF35" s="3" t="inlineStr">
-        <is>
-          <t>✔ Sent</t>
+      <c r="AF35" s="6" t="inlineStr">
+        <is>
+          <t>✔ Delivered (Clean Inbox)</t>
         </is>
       </c>
       <c r="AG35" s="4" t="inlineStr">
@@ -6563,9 +6581,9 @@
           <t>High-intent signal: actively hiring Specialist, Talent Acquisition Operations. Validated website and LinkedIn. Requires Clay enrichment for verified email.</t>
         </is>
       </c>
-      <c r="AF36" s="3" t="inlineStr">
-        <is>
-          <t>✔ Sent</t>
+      <c r="AF36" s="6" t="inlineStr">
+        <is>
+          <t>✔ Delivered (Clean Inbox)</t>
         </is>
       </c>
       <c r="AG36" s="4" t="inlineStr">
@@ -6731,9 +6749,9 @@
           <t>High-intent signal: actively hiring Talent Acquisition Specialist. Validated website and LinkedIn. Requires Clay enrichment for verified email.</t>
         </is>
       </c>
-      <c r="AF37" s="3" t="inlineStr">
-        <is>
-          <t>✔ Sent</t>
+      <c r="AF37" s="7" t="inlineStr">
+        <is>
+          <t>❌ Bounced (Address Not Found)</t>
         </is>
       </c>
       <c r="AG37" s="4" t="inlineStr">
@@ -6899,9 +6917,9 @@
           <t>High-intent signal: actively hiring Senior Talent Acquisition Partner. Validated website and LinkedIn. Requires Clay enrichment for verified email.</t>
         </is>
       </c>
-      <c r="AF38" s="3" t="inlineStr">
-        <is>
-          <t>✔ Sent</t>
+      <c r="AF38" s="7" t="inlineStr">
+        <is>
+          <t>❌ Bounced (Address Not Found)</t>
         </is>
       </c>
       <c r="AG38" s="4" t="inlineStr">
@@ -7067,9 +7085,9 @@
           <t>High-intent signal: actively hiring Talent Acquisition Partner. Validated website and LinkedIn. Requires Clay enrichment for verified email.</t>
         </is>
       </c>
-      <c r="AF39" s="3" t="inlineStr">
-        <is>
-          <t>✔ Sent</t>
+      <c r="AF39" s="7" t="inlineStr">
+        <is>
+          <t>❌ Bounced (Address Not Found)</t>
         </is>
       </c>
       <c r="AG39" s="4" t="inlineStr">
@@ -7235,9 +7253,9 @@
           <t>High-intent signal: actively hiring Associate - Talent Acquisition Recruiter. Validated website and LinkedIn. Requires Clay enrichment for verified email.</t>
         </is>
       </c>
-      <c r="AF40" s="3" t="inlineStr">
-        <is>
-          <t>✔ Sent</t>
+      <c r="AF40" s="7" t="inlineStr">
+        <is>
+          <t>❌ Bounced (Address Not Found)</t>
         </is>
       </c>
       <c r="AG40" s="4" t="inlineStr">
@@ -7403,9 +7421,9 @@
           <t>High-intent signal: actively hiring Assistant Manager, Talent Acquisition. Validated website and LinkedIn. Requires Clay enrichment for verified email.</t>
         </is>
       </c>
-      <c r="AF41" s="3" t="inlineStr">
-        <is>
-          <t>✔ Sent</t>
+      <c r="AF41" s="6" t="inlineStr">
+        <is>
+          <t>✔ Delivered (Clean Inbox)</t>
         </is>
       </c>
       <c r="AG41" s="4" t="inlineStr">
@@ -7571,9 +7589,9 @@
           <t>High-intent signal: actively hiring Talent Acquisition Partner. Validated website and LinkedIn. Requires Clay enrichment for verified email.</t>
         </is>
       </c>
-      <c r="AF42" s="3" t="inlineStr">
-        <is>
-          <t>✔ Sent</t>
+      <c r="AF42" s="7" t="inlineStr">
+        <is>
+          <t>❌ Bounced (Address Not Found)</t>
         </is>
       </c>
       <c r="AG42" s="4" t="inlineStr">
@@ -7739,9 +7757,9 @@
           <t>High-intent signal: actively hiring Talent Acquisition Specialist, Americas. Validated website and LinkedIn. Requires Clay enrichment for verified email.</t>
         </is>
       </c>
-      <c r="AF43" s="3" t="inlineStr">
-        <is>
-          <t>✔ Sent</t>
+      <c r="AF43" s="6" t="inlineStr">
+        <is>
+          <t>✔ Delivered (Clean Inbox)</t>
         </is>
       </c>
       <c r="AG43" s="4" t="inlineStr">
@@ -7907,9 +7925,9 @@
           <t>High-intent signal: actively hiring Talent Acquisition Specialist. Validated website and LinkedIn. Requires Clay enrichment for verified email.</t>
         </is>
       </c>
-      <c r="AF44" s="3" t="inlineStr">
-        <is>
-          <t>✔ Sent</t>
+      <c r="AF44" s="6" t="inlineStr">
+        <is>
+          <t>✔ Delivered (Clean Inbox)</t>
         </is>
       </c>
       <c r="AG44" s="4" t="inlineStr">
@@ -8075,9 +8093,9 @@
           <t>High-intent signal: actively hiring Talent Acquisition Specialist. Validated website and LinkedIn. Requires Clay enrichment for verified email.</t>
         </is>
       </c>
-      <c r="AF45" s="3" t="inlineStr">
-        <is>
-          <t>✔ Sent</t>
+      <c r="AF45" s="6" t="inlineStr">
+        <is>
+          <t>✔ Delivered (Clean Inbox)</t>
         </is>
       </c>
       <c r="AG45" s="4" t="inlineStr">
@@ -8243,9 +8261,9 @@
           <t>High-intent signal: actively hiring Talent Acquisition Specialist. Validated website and LinkedIn. Requires Clay enrichment for verified email.</t>
         </is>
       </c>
-      <c r="AF46" s="3" t="inlineStr">
-        <is>
-          <t>✔ Sent</t>
+      <c r="AF46" s="6" t="inlineStr">
+        <is>
+          <t>✔ Delivered (Clean Inbox)</t>
         </is>
       </c>
       <c r="AG46" s="4" t="inlineStr">
@@ -8411,9 +8429,9 @@
           <t>High-intent signal: actively hiring Manager, Talent Acquisition Corporate. Validated website and LinkedIn. Requires Clay enrichment for verified email.</t>
         </is>
       </c>
-      <c r="AF47" s="3" t="inlineStr">
-        <is>
-          <t>✔ Sent</t>
+      <c r="AF47" s="7" t="inlineStr">
+        <is>
+          <t>❌ Bounced (Address Not Found)</t>
         </is>
       </c>
       <c r="AG47" s="4" t="inlineStr">
@@ -8579,9 +8597,9 @@
           <t>High-intent signal: actively hiring Talent Acquisition Specialist, Americas. Validated website and LinkedIn. Requires Clay enrichment for verified email.</t>
         </is>
       </c>
-      <c r="AF48" s="3" t="inlineStr">
-        <is>
-          <t>✔ Sent</t>
+      <c r="AF48" s="6" t="inlineStr">
+        <is>
+          <t>✔ Delivered (Clean Inbox)</t>
         </is>
       </c>
       <c r="AG48" s="4" t="inlineStr">
@@ -8747,9 +8765,9 @@
           <t>High-intent signal: actively hiring Store Talent Acquisition Manager. Validated website and LinkedIn. Requires Clay enrichment for verified email.</t>
         </is>
       </c>
-      <c r="AF49" s="3" t="inlineStr">
-        <is>
-          <t>✔ Sent</t>
+      <c r="AF49" s="7" t="inlineStr">
+        <is>
+          <t>❌ Bounced (Address Not Found)</t>
         </is>
       </c>
       <c r="AG49" s="4" t="inlineStr">
@@ -8915,9 +8933,9 @@
           <t>High-intent signal: actively hiring Talent Acquisition Specialist / HR. Validated website and LinkedIn. Requires Clay enrichment for verified email.</t>
         </is>
       </c>
-      <c r="AF50" s="3" t="inlineStr">
-        <is>
-          <t>✔ Sent</t>
+      <c r="AF50" s="6" t="inlineStr">
+        <is>
+          <t>✔ Delivered (Clean Inbox)</t>
         </is>
       </c>
       <c r="AG50" s="4" t="inlineStr">
@@ -9083,9 +9101,9 @@
           <t>High-intent signal: actively hiring Talent Acquisition Specialist. Validated website and LinkedIn. Requires Clay enrichment for verified email.</t>
         </is>
       </c>
-      <c r="AF51" s="3" t="inlineStr">
-        <is>
-          <t>✔ Sent</t>
+      <c r="AF51" s="7" t="inlineStr">
+        <is>
+          <t>❌ Bounced (Address Not Found)</t>
         </is>
       </c>
       <c r="AG51" s="4" t="inlineStr">
@@ -9251,9 +9269,9 @@
           <t>High-intent signal: actively hiring Talent Acquisition Partner. Validated website and LinkedIn. Requires Clay enrichment for verified email.</t>
         </is>
       </c>
-      <c r="AF52" s="3" t="inlineStr">
-        <is>
-          <t>✔ Sent</t>
+      <c r="AF52" s="7" t="inlineStr">
+        <is>
+          <t>❌ Bounced (Address Not Found)</t>
         </is>
       </c>
       <c r="AG52" s="4" t="inlineStr">
@@ -9587,9 +9605,9 @@
           <t>High-intent signal: actively hiring Senior Talent Acquisition Specialist. Validated website and LinkedIn. Requires Clay enrichment for verified email.</t>
         </is>
       </c>
-      <c r="AF54" s="3" t="inlineStr">
-        <is>
-          <t>✔ Sent</t>
+      <c r="AF54" s="7" t="inlineStr">
+        <is>
+          <t>❌ Bounced (Address Not Found)</t>
         </is>
       </c>
       <c r="AG54" s="4" t="inlineStr">
@@ -9755,9 +9773,9 @@
           <t>High-intent signal: actively hiring Talent Acquisition Specialist. Validated website and LinkedIn. Requires Clay enrichment for verified email.</t>
         </is>
       </c>
-      <c r="AF55" s="3" t="inlineStr">
-        <is>
-          <t>✔ Sent</t>
+      <c r="AF55" s="6" t="inlineStr">
+        <is>
+          <t>✔ Delivered (Clean Inbox)</t>
         </is>
       </c>
       <c r="AG55" s="4" t="inlineStr">
@@ -9923,9 +9941,9 @@
           <t>High-intent signal: actively hiring Talent Acquisition Specialist. Validated website and LinkedIn. Requires Clay enrichment for verified email.</t>
         </is>
       </c>
-      <c r="AF56" s="3" t="inlineStr">
-        <is>
-          <t>✔ Sent</t>
+      <c r="AF56" s="6" t="inlineStr">
+        <is>
+          <t>✔ Delivered (Clean Inbox)</t>
         </is>
       </c>
       <c r="AG56" s="4" t="inlineStr">
@@ -10091,9 +10109,9 @@
           <t>High-intent signal: actively hiring Talent Acquisition / Recruiting Specialist. Validated website and LinkedIn. Requires Clay enrichment for verified email.</t>
         </is>
       </c>
-      <c r="AF57" s="3" t="inlineStr">
-        <is>
-          <t>✔ Sent</t>
+      <c r="AF57" s="7" t="inlineStr">
+        <is>
+          <t>❌ Bounced (Address Not Found)</t>
         </is>
       </c>
       <c r="AG57" s="4" t="inlineStr">
@@ -10259,9 +10277,9 @@
           <t>High-intent signal: actively hiring Specialist, Talent Acquisition Operations. Validated website and LinkedIn. Requires Clay enrichment for verified email.</t>
         </is>
       </c>
-      <c r="AF58" s="3" t="inlineStr">
-        <is>
-          <t>✔ Sent</t>
+      <c r="AF58" s="6" t="inlineStr">
+        <is>
+          <t>✔ Delivered (Clean Inbox)</t>
         </is>
       </c>
       <c r="AG58" s="4" t="inlineStr">
@@ -10427,9 +10445,9 @@
           <t>High-intent signal: actively hiring Talent Acquisition Sourcing Specialist. Validated website and LinkedIn. Requires Clay enrichment for verified email.</t>
         </is>
       </c>
-      <c r="AF59" s="3" t="inlineStr">
-        <is>
-          <t>✔ Sent</t>
+      <c r="AF59" s="7" t="inlineStr">
+        <is>
+          <t>❌ Bounced (Address Not Found)</t>
         </is>
       </c>
       <c r="AG59" s="4" t="inlineStr">
@@ -10595,9 +10613,9 @@
           <t>High-intent signal: actively hiring Network Talent Acquisition Sourcing Specialist. Validated website and LinkedIn. Requires Clay enrichment for verified email.</t>
         </is>
       </c>
-      <c r="AF60" s="3" t="inlineStr">
-        <is>
-          <t>✔ Sent</t>
+      <c r="AF60" s="7" t="inlineStr">
+        <is>
+          <t>❌ Bounced (Address Not Found)</t>
         </is>
       </c>
       <c r="AG60" s="4" t="inlineStr">
@@ -10931,9 +10949,9 @@
           <t>High-intent signal: actively hiring Technical and Customer Experience Advisor. Validated website and LinkedIn. Requires Clay enrichment for verified email.</t>
         </is>
       </c>
-      <c r="AF62" s="3" t="inlineStr">
-        <is>
-          <t>✔ Sent</t>
+      <c r="AF62" s="7" t="inlineStr">
+        <is>
+          <t>❌ Bounced (Address Not Found)</t>
         </is>
       </c>
       <c r="AG62" s="4" t="inlineStr">
@@ -11099,9 +11117,9 @@
           <t>High-intent signal: actively hiring Recruiting Specialist. Validated website and LinkedIn. Requires Clay enrichment for verified email.</t>
         </is>
       </c>
-      <c r="AF63" s="3" t="inlineStr">
-        <is>
-          <t>✔ Sent</t>
+      <c r="AF63" s="6" t="inlineStr">
+        <is>
+          <t>✔ Delivered (Clean Inbox)</t>
         </is>
       </c>
       <c r="AG63" s="4" t="inlineStr">
@@ -11267,9 +11285,9 @@
           <t>High-intent signal: actively hiring Senior Recruiter. Validated website and LinkedIn. Requires Clay enrichment for verified email.</t>
         </is>
       </c>
-      <c r="AF64" s="3" t="inlineStr">
-        <is>
-          <t>✔ Sent</t>
+      <c r="AF64" s="6" t="inlineStr">
+        <is>
+          <t>✔ Delivered (Clean Inbox)</t>
         </is>
       </c>
       <c r="AG64" s="4" t="inlineStr">
@@ -11435,9 +11453,9 @@
           <t>High-intent signal: actively hiring Email Marketing &amp; Lifecycle Manager. Validated website and LinkedIn. Requires Clay enrichment for verified email.</t>
         </is>
       </c>
-      <c r="AF65" s="3" t="inlineStr">
-        <is>
-          <t>✔ Sent</t>
+      <c r="AF65" s="7" t="inlineStr">
+        <is>
+          <t>❌ Bounced (Address Not Found)</t>
         </is>
       </c>
       <c r="AG65" s="4" t="inlineStr">
@@ -11603,9 +11621,9 @@
           <t>High-intent signal: actively hiring Recruiter. Validated website and LinkedIn. Requires Clay enrichment for verified email.</t>
         </is>
       </c>
-      <c r="AF66" s="3" t="inlineStr">
-        <is>
-          <t>✔ Sent</t>
+      <c r="AF66" s="6" t="inlineStr">
+        <is>
+          <t>✔ Delivered (Clean Inbox)</t>
         </is>
       </c>
       <c r="AG66" s="4" t="inlineStr">
@@ -11771,9 +11789,9 @@
           <t>High-intent signal: actively hiring Support Operations Manager. Validated website and LinkedIn. Requires Clay enrichment for verified email.</t>
         </is>
       </c>
-      <c r="AF67" s="3" t="inlineStr">
-        <is>
-          <t>✔ Sent</t>
+      <c r="AF67" s="7" t="inlineStr">
+        <is>
+          <t>❌ Bounced (Address Not Found)</t>
         </is>
       </c>
       <c r="AG67" s="4" t="inlineStr">
@@ -11939,9 +11957,9 @@
           <t>High-intent signal: actively hiring CRM Executive / CRM Specialist. Validated website and LinkedIn. Requires Clay enrichment for verified email.</t>
         </is>
       </c>
-      <c r="AF68" s="3" t="inlineStr">
-        <is>
-          <t>✔ Sent</t>
+      <c r="AF68" s="7" t="inlineStr">
+        <is>
+          <t>❌ Bounced (Address Not Found)</t>
         </is>
       </c>
       <c r="AG68" s="4" t="inlineStr">
@@ -12107,9 +12125,9 @@
           <t>High-intent signal: actively hiring Regional Recruiter. Validated website and LinkedIn. Requires Clay enrichment for verified email.</t>
         </is>
       </c>
-      <c r="AF69" s="3" t="inlineStr">
-        <is>
-          <t>✔ Sent</t>
+      <c r="AF69" s="7" t="inlineStr">
+        <is>
+          <t>❌ Bounced (Address Not Found)</t>
         </is>
       </c>
       <c r="AG69" s="4" t="inlineStr">
@@ -12275,9 +12293,9 @@
           <t>High-intent signal: actively hiring Product Operations Manager, AI &amp; Systems. Validated website and LinkedIn. Requires Clay enrichment for verified email.</t>
         </is>
       </c>
-      <c r="AF70" s="3" t="inlineStr">
-        <is>
-          <t>✔ Sent</t>
+      <c r="AF70" s="7" t="inlineStr">
+        <is>
+          <t>❌ Bounced (Address Not Found)</t>
         </is>
       </c>
       <c r="AG70" s="4" t="inlineStr">
@@ -12443,9 +12461,9 @@
           <t>High-intent signal: actively hiring Front Office Receptionist. Validated website and LinkedIn. Requires Clay enrichment for verified email.</t>
         </is>
       </c>
-      <c r="AF71" s="3" t="inlineStr">
-        <is>
-          <t>✔ Sent</t>
+      <c r="AF71" s="6" t="inlineStr">
+        <is>
+          <t>✔ Delivered (Clean Inbox)</t>
         </is>
       </c>
       <c r="AG71" s="4" t="inlineStr">
@@ -12611,9 +12629,9 @@
           <t>High-intent signal: actively hiring Recruiter. Validated website and LinkedIn. Requires Clay enrichment for verified email.</t>
         </is>
       </c>
-      <c r="AF72" s="3" t="inlineStr">
-        <is>
-          <t>✔ Sent</t>
+      <c r="AF72" s="6" t="inlineStr">
+        <is>
+          <t>✔ Delivered (Clean Inbox)</t>
         </is>
       </c>
       <c r="AG72" s="4" t="inlineStr">
@@ -12779,9 +12797,9 @@
           <t>High-intent signal: actively hiring Recruiter. Validated website and LinkedIn. Requires Clay enrichment for verified email.</t>
         </is>
       </c>
-      <c r="AF73" s="3" t="inlineStr">
-        <is>
-          <t>✔ Sent</t>
+      <c r="AF73" s="7" t="inlineStr">
+        <is>
+          <t>❌ Bounced (Address Not Found)</t>
         </is>
       </c>
       <c r="AG73" s="4" t="inlineStr">
@@ -12947,9 +12965,9 @@
           <t>High-intent signal: actively hiring Property Sales Representative. Validated website and LinkedIn. Requires Clay enrichment for verified email.</t>
         </is>
       </c>
-      <c r="AF74" s="3" t="inlineStr">
-        <is>
-          <t>✔ Sent</t>
+      <c r="AF74" s="6" t="inlineStr">
+        <is>
+          <t>✔ Delivered (Clean Inbox)</t>
         </is>
       </c>
       <c r="AG74" s="4" t="inlineStr">
@@ -13115,9 +13133,9 @@
           <t>High-intent signal: actively hiring Customer Support Executive. Validated website and LinkedIn. Requires Clay enrichment for verified email.</t>
         </is>
       </c>
-      <c r="AF75" s="3" t="inlineStr">
-        <is>
-          <t>✔ Sent</t>
+      <c r="AF75" s="6" t="inlineStr">
+        <is>
+          <t>✔ Delivered (Clean Inbox)</t>
         </is>
       </c>
       <c r="AG75" s="4" t="inlineStr">
@@ -13283,9 +13301,9 @@
           <t>High-intent signal: actively hiring Patient Relations Executive. Validated website and LinkedIn. Requires Clay enrichment for verified email.</t>
         </is>
       </c>
-      <c r="AF76" s="3" t="inlineStr">
-        <is>
-          <t>✔ Sent</t>
+      <c r="AF76" s="7" t="inlineStr">
+        <is>
+          <t>❌ Bounced (Address Not Found)</t>
         </is>
       </c>
       <c r="AG76" s="4" t="inlineStr">
@@ -13451,9 +13469,9 @@
           <t>High-intent signal: actively hiring Corporate Recruiter. Validated website and LinkedIn. Requires Clay enrichment for verified email.</t>
         </is>
       </c>
-      <c r="AF77" s="3" t="inlineStr">
-        <is>
-          <t>✔ Sent</t>
+      <c r="AF77" s="7" t="inlineStr">
+        <is>
+          <t>❌ Bounced (Address Not Found)</t>
         </is>
       </c>
       <c r="AG77" s="4" t="inlineStr">
@@ -13619,9 +13637,9 @@
           <t>High-intent signal: actively hiring Customer Success Representative Luxury. Validated website and LinkedIn. Requires Clay enrichment for verified email.</t>
         </is>
       </c>
-      <c r="AF78" s="3" t="inlineStr">
-        <is>
-          <t>✔ Sent</t>
+      <c r="AF78" s="7" t="inlineStr">
+        <is>
+          <t>❌ Bounced (Address Not Found)</t>
         </is>
       </c>
       <c r="AG78" s="4" t="inlineStr">
@@ -13787,9 +13805,9 @@
           <t>High-intent signal: actively hiring Customer Success Manager E-commerce. Validated website and LinkedIn. Requires Clay enrichment for verified email.</t>
         </is>
       </c>
-      <c r="AF79" s="3" t="inlineStr">
-        <is>
-          <t>✔ Sent</t>
+      <c r="AF79" s="7" t="inlineStr">
+        <is>
+          <t>❌ Bounced (Address Not Found)</t>
         </is>
       </c>
       <c r="AG79" s="4" t="inlineStr">
@@ -13955,9 +13973,9 @@
           <t>High-intent signal: actively hiring Real Estate Sales Executive. Validated website and LinkedIn. Requires Clay enrichment for verified email.</t>
         </is>
       </c>
-      <c r="AF80" s="3" t="inlineStr">
-        <is>
-          <t>✔ Sent</t>
+      <c r="AF80" s="7" t="inlineStr">
+        <is>
+          <t>❌ Bounced (Address Not Found)</t>
         </is>
       </c>
       <c r="AG80" s="4" t="inlineStr">
@@ -14123,9 +14141,9 @@
           <t>High-intent signal: actively hiring Customer Support Representative E-commerce/DTC. Validated website and LinkedIn. Requires Clay enrichment for verified email.</t>
         </is>
       </c>
-      <c r="AF81" s="3" t="inlineStr">
-        <is>
-          <t>✔ Sent</t>
+      <c r="AF81" s="7" t="inlineStr">
+        <is>
+          <t>❌ Bounced (Address Not Found)</t>
         </is>
       </c>
       <c r="AG81" s="4" t="inlineStr">
@@ -14291,9 +14309,9 @@
           <t>High-intent signal: actively hiring Technical Recruiter. Validated website and LinkedIn. Requires Clay enrichment for verified email.</t>
         </is>
       </c>
-      <c r="AF82" s="3" t="inlineStr">
-        <is>
-          <t>✔ Sent</t>
+      <c r="AF82" s="7" t="inlineStr">
+        <is>
+          <t>❌ Bounced (Address Not Found)</t>
         </is>
       </c>
       <c r="AG82" s="4" t="inlineStr">
@@ -14459,9 +14477,9 @@
           <t>High-intent signal: actively hiring Talent Partner. Validated website and LinkedIn. Requires Clay enrichment for verified email.</t>
         </is>
       </c>
-      <c r="AF83" s="3" t="inlineStr">
-        <is>
-          <t>✔ Sent</t>
+      <c r="AF83" s="7" t="inlineStr">
+        <is>
+          <t>❌ Bounced (Address Not Found)</t>
         </is>
       </c>
       <c r="AG83" s="4" t="inlineStr">
@@ -14627,9 +14645,9 @@
           <t>High-intent signal: actively hiring E-Commerce Customer Support Specialist. Validated website and LinkedIn. Requires Clay enrichment for verified email.</t>
         </is>
       </c>
-      <c r="AF84" s="3" t="inlineStr">
-        <is>
-          <t>✔ Sent</t>
+      <c r="AF84" s="6" t="inlineStr">
+        <is>
+          <t>✔ Delivered (Clean Inbox)</t>
         </is>
       </c>
       <c r="AG84" s="4" t="inlineStr">
@@ -14795,9 +14813,9 @@
           <t>High-intent signal: actively hiring People &amp; Talent Specialist. Validated website and LinkedIn. Requires Clay enrichment for verified email.</t>
         </is>
       </c>
-      <c r="AF85" s="3" t="inlineStr">
-        <is>
-          <t>✔ Sent</t>
+      <c r="AF85" s="7" t="inlineStr">
+        <is>
+          <t>❌ Bounced (Address Not Found)</t>
         </is>
       </c>
       <c r="AG85" s="4" t="inlineStr">
@@ -14963,9 +14981,9 @@
           <t>High-intent signal: actively hiring Medical Billing &amp; Admin Coordinator. Validated website and LinkedIn. Requires Clay enrichment for verified email.</t>
         </is>
       </c>
-      <c r="AF86" s="3" t="inlineStr">
-        <is>
-          <t>✔ Sent</t>
+      <c r="AF86" s="6" t="inlineStr">
+        <is>
+          <t>✔ Delivered (Clean Inbox)</t>
         </is>
       </c>
       <c r="AG86" s="4" t="inlineStr">
@@ -15131,9 +15149,9 @@
           <t>High-intent signal: actively hiring Sourcing Recruiter. Validated website and LinkedIn. Requires Clay enrichment for verified email.</t>
         </is>
       </c>
-      <c r="AF87" s="3" t="inlineStr">
-        <is>
-          <t>✔ Sent</t>
+      <c r="AF87" s="7" t="inlineStr">
+        <is>
+          <t>❌ Bounced (Address Not Found)</t>
         </is>
       </c>
       <c r="AG87" s="4" t="inlineStr">
@@ -15299,9 +15317,9 @@
           <t>High-intent signal: actively hiring Technical Recruiter, Early Career. Validated website and LinkedIn. Requires Clay enrichment for verified email.</t>
         </is>
       </c>
-      <c r="AF88" s="3" t="inlineStr">
-        <is>
-          <t>✔ Sent</t>
+      <c r="AF88" s="7" t="inlineStr">
+        <is>
+          <t>❌ Bounced (Address Not Found)</t>
         </is>
       </c>
       <c r="AG88" s="4" t="inlineStr">
@@ -15467,9 +15485,9 @@
           <t>High-intent signal: actively hiring Associate Campus Recruiter Hybrid. Validated website and LinkedIn. Requires Clay enrichment for verified email.</t>
         </is>
       </c>
-      <c r="AF89" s="3" t="inlineStr">
-        <is>
-          <t>✔ Sent</t>
+      <c r="AF89" s="7" t="inlineStr">
+        <is>
+          <t>❌ Bounced (Address Not Found)</t>
         </is>
       </c>
       <c r="AG89" s="4" t="inlineStr">
@@ -15635,9 +15653,9 @@
           <t>High-intent signal: actively hiring Recruiter. Validated website and LinkedIn. Requires Clay enrichment for verified email.</t>
         </is>
       </c>
-      <c r="AF90" s="3" t="inlineStr">
-        <is>
-          <t>✔ Sent</t>
+      <c r="AF90" s="7" t="inlineStr">
+        <is>
+          <t>❌ Bounced (Address Not Found)</t>
         </is>
       </c>
       <c r="AG90" s="4" t="inlineStr">
@@ -15803,9 +15821,9 @@
           <t>High-intent signal: actively hiring Lifecycle CRM Marketing Manager. Validated website and LinkedIn. Requires Clay enrichment for verified email.</t>
         </is>
       </c>
-      <c r="AF91" s="3" t="inlineStr">
-        <is>
-          <t>✔ Sent</t>
+      <c r="AF91" s="7" t="inlineStr">
+        <is>
+          <t>❌ Bounced (Address Not Found)</t>
         </is>
       </c>
       <c r="AG91" s="4" t="inlineStr">
@@ -15971,9 +15989,9 @@
           <t>High-intent signal: actively hiring CRM Campaign Manager. Validated website and LinkedIn. Requires Clay enrichment for verified email.</t>
         </is>
       </c>
-      <c r="AF92" s="3" t="inlineStr">
-        <is>
-          <t>✔ Sent</t>
+      <c r="AF92" s="7" t="inlineStr">
+        <is>
+          <t>❌ Bounced (Address Not Found)</t>
         </is>
       </c>
       <c r="AG92" s="4" t="inlineStr">
@@ -16139,9 +16157,9 @@
           <t>High-intent signal: actively hiring Real Estate Sales Associate. Validated website and LinkedIn. Requires Clay enrichment for verified email.</t>
         </is>
       </c>
-      <c r="AF93" s="3" t="inlineStr">
-        <is>
-          <t>✔ Sent</t>
+      <c r="AF93" s="6" t="inlineStr">
+        <is>
+          <t>✔ Delivered (Clean Inbox)</t>
         </is>
       </c>
       <c r="AG93" s="4" t="inlineStr">
@@ -16307,9 +16325,9 @@
           <t>High-intent signal: actively hiring Executive Recruiting Coordinator. Validated website and LinkedIn. Requires Clay enrichment for verified email.</t>
         </is>
       </c>
-      <c r="AF94" s="3" t="inlineStr">
-        <is>
-          <t>✔ Sent</t>
+      <c r="AF94" s="6" t="inlineStr">
+        <is>
+          <t>✔ Delivered (Clean Inbox)</t>
         </is>
       </c>
       <c r="AG94" s="4" t="inlineStr">
@@ -16475,9 +16493,9 @@
           <t>High-intent signal: actively hiring Technical Recruiter AI-Savvy. Validated website and LinkedIn. Requires Clay enrichment for verified email.</t>
         </is>
       </c>
-      <c r="AF95" s="3" t="inlineStr">
-        <is>
-          <t>✔ Sent</t>
+      <c r="AF95" s="7" t="inlineStr">
+        <is>
+          <t>❌ Bounced (Address Not Found)</t>
         </is>
       </c>
       <c r="AG95" s="4" t="inlineStr">
@@ -16643,9 +16661,9 @@
           <t>High-intent signal: actively hiring Senior Knowledge Management Specialist. Validated website and LinkedIn. Requires Clay enrichment for verified email.</t>
         </is>
       </c>
-      <c r="AF96" s="3" t="inlineStr">
-        <is>
-          <t>✔ Sent</t>
+      <c r="AF96" s="6" t="inlineStr">
+        <is>
+          <t>✔ Delivered (Clean Inbox)</t>
         </is>
       </c>
       <c r="AG96" s="4" t="inlineStr">
@@ -16811,9 +16829,9 @@
           <t>High-intent signal: actively hiring Staff Business Operations Manager, GTM. Validated website and LinkedIn. Requires Clay enrichment for verified email.</t>
         </is>
       </c>
-      <c r="AF97" s="3" t="inlineStr">
-        <is>
-          <t>✔ Sent</t>
+      <c r="AF97" s="7" t="inlineStr">
+        <is>
+          <t>❌ Bounced (Address Not Found)</t>
         </is>
       </c>
       <c r="AG97" s="4" t="inlineStr">
@@ -16979,9 +16997,9 @@
           <t>High-intent signal: actively hiring Real Estate CRM Executive. Validated website and LinkedIn. Requires Clay enrichment for verified email.</t>
         </is>
       </c>
-      <c r="AF98" s="3" t="inlineStr">
-        <is>
-          <t>✔ Sent</t>
+      <c r="AF98" s="7" t="inlineStr">
+        <is>
+          <t>❌ Bounced (Address Not Found)</t>
         </is>
       </c>
       <c r="AG98" s="4" t="inlineStr">
@@ -17315,9 +17333,9 @@
           <t>High-intent signal: actively hiring Sourcing Recruiter. Validated website and LinkedIn. Requires Clay enrichment for verified email.</t>
         </is>
       </c>
-      <c r="AF100" s="3" t="inlineStr">
-        <is>
-          <t>✔ Sent</t>
+      <c r="AF100" s="6" t="inlineStr">
+        <is>
+          <t>✔ Delivered (Clean Inbox)</t>
         </is>
       </c>
       <c r="AG100" s="4" t="inlineStr">
@@ -17483,9 +17501,9 @@
           <t>High-intent signal: actively hiring Hourly Recruiter. Validated website and LinkedIn. Requires Clay enrichment for verified email.</t>
         </is>
       </c>
-      <c r="AF101" s="3" t="inlineStr">
-        <is>
-          <t>✔ Sent</t>
+      <c r="AF101" s="6" t="inlineStr">
+        <is>
+          <t>✔ Delivered (Clean Inbox)</t>
         </is>
       </c>
       <c r="AG101" s="4" t="inlineStr">

</xml_diff>